<commit_message>
Tareas 231, 51 y 238 Percepciones
</commit_message>
<xml_diff>
--- a/Plantilla/TemplateFacturas.xlsx
+++ b/Plantilla/TemplateFacturas.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="21929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28526"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\stambour\OneDrive - DXC Production\Personal\Desarrollo\Repos\Cinderella\Plantilla\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://dxcportal-my.sharepoint.com/personal/santiago_tambour_dxc_com/Documents/Personal/Desarrollo/Repos/Cinderella/Plantilla/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="25" documentId="11_D91601F0DED5E7358A217455409C7F49F501C076" xr6:coauthVersionLast="44" xr6:coauthVersionMax="44" xr10:uidLastSave="{D5C3CBA1-A980-4214-B78B-329D616DFEFB}"/>
+  <xr:revisionPtr revIDLastSave="28" documentId="11_D91601F0DED5E7358A217455409C7F49F501C076" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{3EF6294F-6DA2-4658-8277-D868E0009FA3}"/>
   <bookViews>
-    <workbookView xWindow="3735" yWindow="3075" windowWidth="21600" windowHeight="11385" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-135" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Facturas" sheetId="2" r:id="rId1"/>
@@ -29,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="13" uniqueCount="13">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14" uniqueCount="14">
   <si>
     <t>Sucursal:</t>
   </si>
@@ -68,6 +68,9 @@
   </si>
   <si>
     <t>Total</t>
+  </si>
+  <si>
+    <t>Provincia</t>
   </si>
 </sst>
 </file>
@@ -469,28 +472,28 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:L5"/>
+  <dimension ref="A1:M5"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="15.7109375" style="22" customWidth="1"/>
     <col min="2" max="2" width="15.7109375" style="17" customWidth="1"/>
     <col min="3" max="3" width="15.7109375" style="12" customWidth="1"/>
     <col min="4" max="4" width="15.7109375" customWidth="1"/>
-    <col min="5" max="9" width="15.7109375" style="18" customWidth="1"/>
-    <col min="10" max="12" width="15.7109375" style="5" customWidth="1"/>
+    <col min="5" max="10" width="15.7109375" style="18" customWidth="1"/>
+    <col min="11" max="13" width="15.7109375" style="5" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A1" s="25" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="13"/>
       <c r="C1"/>
     </row>
-    <row r="2" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:13" x14ac:dyDescent="0.25">
       <c r="C2"/>
     </row>
-    <row r="3" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A3" s="4" t="s">
         <v>9</v>
       </c>
@@ -518,17 +521,20 @@
       <c r="I3" s="19" t="s">
         <v>8</v>
       </c>
-      <c r="J3" s="6" t="s">
+      <c r="J3" s="19" t="s">
+        <v>13</v>
+      </c>
+      <c r="K3" s="6" t="s">
         <v>10</v>
       </c>
-      <c r="K3" s="6" t="s">
+      <c r="L3" s="6" t="s">
         <v>11</v>
       </c>
-      <c r="L3" s="6" t="s">
+      <c r="M3" s="6" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="4" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A4" s="23"/>
       <c r="B4" s="15"/>
       <c r="C4" s="10"/>
@@ -538,11 +544,12 @@
       <c r="G4" s="20"/>
       <c r="H4" s="20"/>
       <c r="I4" s="20"/>
-      <c r="J4" s="7"/>
+      <c r="J4" s="20"/>
       <c r="K4" s="7"/>
       <c r="L4" s="7"/>
+      <c r="M4" s="7"/>
     </row>
-    <row r="5" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A5" s="24"/>
       <c r="B5" s="16"/>
       <c r="C5" s="11"/>
@@ -552,9 +559,10 @@
       <c r="G5" s="21"/>
       <c r="H5" s="21"/>
       <c r="I5" s="21"/>
-      <c r="J5" s="8"/>
+      <c r="J5" s="21"/>
       <c r="K5" s="8"/>
       <c r="L5" s="8"/>
+      <c r="M5" s="8"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>